<commit_message>
updating schedule pages and presentations with live links
</commit_message>
<xml_diff>
--- a/AEDU event schedule.xlsx
+++ b/AEDU event schedule.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\jasonayoder\git_repos\alife-edu.github.io\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{753220CD-C3DF-4FF7-A337-DC0167582BD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CD4951B-DD13-42B4-B218-7CA035B07EFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-1485" yWindow="-16665" windowWidth="34335" windowHeight="14280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-3900" yWindow="-18405" windowWidth="34335" windowHeight="14280" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="N. America" sheetId="1" r:id="rId1"/>
     <sheet name="JPAsia (Compressed)" sheetId="3" r:id="rId2"/>
+    <sheet name="west-day1-videos" sheetId="4" r:id="rId3"/>
+    <sheet name="west-day2-videos" sheetId="5" r:id="rId4"/>
+    <sheet name="east-videos" sheetId="6" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="113">
   <si>
     <t>Day 1</t>
   </si>
@@ -310,12 +313,189 @@
       <t>All participants + Speakers</t>
     </r>
   </si>
+  <si>
+    <t>Topic</t>
+  </si>
+  <si>
+    <t>Video Link</t>
+  </si>
+  <si>
+    <t>Talk by Imy Khan -
+Artificial Life is everywhere: 
+So why is it so hard to teach?</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Talk by Q. Tyrell Davis:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Reaching (for) Critical Maths</t>
+    </r>
+  </si>
+  <si>
+    <t>Day 1 Wrap Up and Feedback Exchange Intro</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=z-lJFxy4yTw</t>
+  </si>
+  <si>
+    <t>Small Group Feedback on __
+3x15 minutes / 4x10
+(NOT RECORDED)</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=z-lJFxy4yTw&amp;t=69s</t>
+  </si>
+  <si>
+    <t>Talk by Jason Yoder:
+Creating Space to Grow Intrinsic Motivation for ALife</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=z-lJFxy4yTw&amp;t=235s</t>
+  </si>
+  <si>
+    <t>Talk by Anya Vostinar:
+Grading as it could be: 
+Aligning Incentives with Intellectual Curiosity</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=z-lJFxy4yTw&amp;t=1607s</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=z-lJFxy4yTw&amp;t=3038s</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=z-lJFxy4yTw&amp;t=4125s</t>
+  </si>
+  <si>
+    <t>Discussion: Future Goals for ALife Educators</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=z-lJFxy4yTw&amp;t=5417s</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=z-lJFxy4yTw&amp;t=7886s</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=z-lJFxy4yTw&amp;t=8270s</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=pJ3Xb_oBrGk</t>
+  </si>
+  <si>
+    <t>- Welcome and introductions</t>
+  </si>
+  <si>
+    <t>topic</t>
+  </si>
+  <si>
+    <t>video link</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=pJ3Xb_oBrGk&amp;t=780s</t>
+  </si>
+  <si>
+    <t>Summary of AEdu - West</t>
+  </si>
+  <si>
+    <t>Bert Chan: "Teaching Cellular Automata"</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=pJ3Xb_oBrGk&amp;t=1033s</t>
+  </si>
+  <si>
+    <t>Takashi Ikegami: "From Parts to Wholes: Teaching ALife through Emergence, Embodiment, and Collective Intelligence"</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=pJ3Xb_oBrGk&amp;t=3418s</t>
+  </si>
+  <si>
+    <t>Keisuke Suzuki: "Understanding by Building: ALife Approaches to Mind, and How We Share Them"</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=pJ3Xb_oBrGk&amp;t=5619s</t>
+  </si>
+  <si>
+    <t>Panel discussion: "Art and Beauty in ALife"</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=pJ3Xb_oBrGk&amp;t=7642s</t>
+  </si>
+  <si>
+    <t>Wrap-up and ALife2026 workshop announcement</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=pJ3Xb_oBrGk&amp;t=10315s</t>
+  </si>
+  <si>
+    <t>Eduardo Izquierdo</t>
+  </si>
+  <si>
+    <t>Stephen Kelley</t>
+  </si>
+  <si>
+    <t>Corne</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=FeQ51wp_Yls</t>
+  </si>
+  <si>
+    <t>Matthew Moreno</t>
+  </si>
+  <si>
+    <t>lightning talks - intro</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=bHGJc1kqtG0&amp;t=0</t>
+  </si>
+  <si>
+    <t>https://youtu.be/bHGJc1kqtG0?si=-vhpk0ne131Huq1w&amp;t=5717</t>
+  </si>
+  <si>
+    <t>https://youtu.be/bHGJc1kqtG0?si=-vhpk0ne131Huq1w&amp;t=6496</t>
+  </si>
+  <si>
+    <t>https://youtu.be/bHGJc1kqtG0?si=-vhpk0ne131Huq1w&amp;t=6888</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=bHGJc1kqtG0&amp;t=971s</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=bHGJc1kqtG0&amp;t=1217s</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=bHGJc1kqtG0&amp;t=2553s</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=bHGJc1kqtG0&amp;t=3034s</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=bHGJc1kqtG0&amp;t=3745s</t>
+  </si>
+  <si>
+    <t>https://youtu.be/bHGJc1kqtG0?si=-vhpk0ne131Huq1w&amp;t=5281</t>
+  </si>
+  <si>
+    <t>https://youtu.be/bHGJc1kqtG0?si=-vhpk0ne131Huq1w&amp;t=5332</t>
+  </si>
+  <si>
+    <t>https://youtu.be/bHGJc1kqtG0?si=-vhpk0ne131Huq1w&amp;t=6143</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -343,8 +523,26 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF065FD4"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF131313"/>
+      <name val="Roboto"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -390,6 +588,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFB4A7D6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -508,10 +724,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -615,8 +832,34 @@
     <xf numFmtId="0" fontId="2" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -630,10 +873,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9744,4 +9983,321 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D96B7CD-AB01-430C-BCD8-94E4CFC44903}">
+  <dimension ref="C1:F15"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="30.88671875" customWidth="1"/>
+    <col min="4" max="4" width="63.6640625" customWidth="1"/>
+    <col min="5" max="5" width="59" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="3:6" ht="13.8" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="3:6" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C2" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="3:6" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C3" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="46" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="4" spans="3:6" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C4" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="38" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="5" spans="3:6" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C5" s="39" t="s">
+        <v>63</v>
+      </c>
+      <c r="D5" s="46" t="s">
+        <v>106</v>
+      </c>
+      <c r="F5" s="46"/>
+    </row>
+    <row r="6" spans="3:6" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C6" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="46" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="7" spans="3:6" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C7" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="46" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="8" spans="3:6" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C8" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="D8" s="46" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="9" spans="3:6" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C9" s="37" t="s">
+        <v>100</v>
+      </c>
+      <c r="D9" s="46" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="10" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C10" s="47" t="s">
+        <v>95</v>
+      </c>
+      <c r="D10" s="46" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="11" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C11" s="47" t="s">
+        <v>96</v>
+      </c>
+      <c r="D11" s="46" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="12" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C12" s="47" t="s">
+        <v>99</v>
+      </c>
+      <c r="D12" s="46" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="13" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C13" s="47" t="s">
+        <v>97</v>
+      </c>
+      <c r="D13" s="46" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="14" spans="3:6" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C14" s="47" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" s="46" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="15" spans="3:6" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C15" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="D15" s="37" t="s">
+        <v>104</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C9" r:id="rId1" location="slide=id.g3e141100d42_0_121" display="https://docs.google.com/presentation/d/12Ev1s7-mrVxJsgGT2Fq4GM7wV4r3ILVERgkX8Rqpixw/edit?slide=id.g3e141100d42_0_121 - slide=id.g3e141100d42_0_121" xr:uid="{2C4FE182-9D74-4EA3-9CFF-9640BBE5F0B1}"/>
+    <hyperlink ref="D13" r:id="rId2" xr:uid="{759901EE-80F2-43D7-84DA-C1611A51C3BD}"/>
+    <hyperlink ref="D3" r:id="rId3" xr:uid="{74BEE726-E2A6-44EF-9739-04852263165B}"/>
+    <hyperlink ref="D11" r:id="rId4" xr:uid="{EEE6E13E-6E00-4E94-A398-9C36C8BDD6AB}"/>
+    <hyperlink ref="D12" r:id="rId5" xr:uid="{084A66EF-1FC6-4109-88A1-581969DAFEAB}"/>
+    <hyperlink ref="D14" r:id="rId6" xr:uid="{2C40C846-8C4C-4638-A7E9-01D7B8EC05AE}"/>
+    <hyperlink ref="D15" r:id="rId7" xr:uid="{A9A5762B-C259-4E70-8C38-6B1C36C2901D}"/>
+    <hyperlink ref="D10" r:id="rId8" xr:uid="{63394D16-FA02-4E62-BCC2-8331A8D83F9B}"/>
+    <hyperlink ref="D9" r:id="rId9" xr:uid="{156BDBD3-AAD8-4120-ABA8-736046480ECB}"/>
+    <hyperlink ref="D4" r:id="rId10" xr:uid="{2BB16030-0AAC-44B2-A8FE-A27DCC5D96DB}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{074D7817-DA02-467D-9FD1-C39A354C8719}">
+  <dimension ref="C3:D12"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="26" customWidth="1"/>
+    <col min="4" max="4" width="33.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="3:4" ht="13.8" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="4" spans="3:4" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C4" s="39" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="41" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5" spans="3:4" ht="53.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C5" s="42" t="s">
+        <v>67</v>
+      </c>
+      <c r="D5" s="41" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" spans="3:4" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C6" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="D6" s="41" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="7" spans="3:4" ht="53.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C7" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="D7" s="41" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" spans="3:4" ht="53.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C8" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="D8" s="41" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="9" spans="3:4" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C9" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="41" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="10" spans="3:4" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C10" s="43" t="s">
+        <v>75</v>
+      </c>
+      <c r="D10" s="41" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11" spans="3:4" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C11" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" s="41" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="12" spans="3:4" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C12" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12" s="41" t="s">
+        <v>78</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D4" r:id="rId1" xr:uid="{8CE7EB96-1479-416E-9708-38743B84EDF4}"/>
+    <hyperlink ref="D5" r:id="rId2" xr:uid="{DB0B1EB7-9F7A-43A5-ADDB-7ED6179756D8}"/>
+    <hyperlink ref="D6" r:id="rId3" xr:uid="{0B6FBA5B-EE05-42B9-A1B6-A47E45146AFB}"/>
+    <hyperlink ref="D7" r:id="rId4" xr:uid="{10BE4241-5A34-4B41-8579-15C8F5955170}"/>
+    <hyperlink ref="D8" r:id="rId5" xr:uid="{C29CADE9-F353-4643-B8F8-3E27DA1CCA1F}"/>
+    <hyperlink ref="D9" r:id="rId6" xr:uid="{ACB2762B-8199-4D1C-9844-BC597600342F}"/>
+    <hyperlink ref="D10" r:id="rId7" xr:uid="{61FC47DF-3FC4-46E8-9CF7-F6CDA428999A}"/>
+    <hyperlink ref="D11" r:id="rId8" xr:uid="{7DB0AC41-F444-44E9-A14E-8805896B18E9}"/>
+    <hyperlink ref="D12" r:id="rId9" xr:uid="{B6BBCB4E-2C1A-499A-B1C7-F1CCF49EE3DB}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C8D369E4-D048-4CB5-9292-EF4445CB1EDB}">
+  <dimension ref="D5:H12"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="51.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="5" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D5" s="40" t="s">
+        <v>81</v>
+      </c>
+      <c r="E5" s="40" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D6" s="45" t="s">
+        <v>80</v>
+      </c>
+      <c r="E6" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="7" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D7" s="45" t="s">
+        <v>84</v>
+      </c>
+      <c r="E7" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="8" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D8" s="45" t="s">
+        <v>85</v>
+      </c>
+      <c r="E8" t="s">
+        <v>86</v>
+      </c>
+      <c r="H8" s="44"/>
+    </row>
+    <row r="9" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D9" t="s">
+        <v>88</v>
+      </c>
+      <c r="E9" s="45" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="10" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D10" t="s">
+        <v>90</v>
+      </c>
+      <c r="E10" s="45" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="11" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D11" t="s">
+        <v>92</v>
+      </c>
+      <c r="E11" s="45" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="12" spans="4:8" x14ac:dyDescent="0.25">
+      <c r="D12" t="s">
+        <v>94</v>
+      </c>
+      <c r="E12" s="45" t="s">
+        <v>93</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>